<commit_message>
Acertos visuais e adição da tela distribuição de lucros
</commit_message>
<xml_diff>
--- a/dist/EDR - DashboardFinanceiro/data/Faturamento Allan.xlsx
+++ b/dist/EDR - DashboardFinanceiro/data/Faturamento Allan.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\GERENCIAL\Centros de Custo\Orçamento 2026\Planilhas - Faturamento Miguel-Bruno\01. Faturamento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB534B9E-0267-4063-AB27-DB81641D19C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E23B1FB3-04BA-4D8D-9F14-AD7F20C90692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9762,7 +9762,7 @@
         <v>61168.24</v>
       </c>
       <c r="E171" s="5">
-        <v>0</v>
+        <v>106396.24</v>
       </c>
       <c r="F171" s="5">
         <v>0</v>
@@ -9792,13 +9792,13 @@
         <v>0</v>
       </c>
       <c r="O171" s="16">
-        <v>152937.9</v>
+        <v>259334.14</v>
       </c>
       <c r="P171" s="17">
-        <v>76468.95</v>
+        <v>86444.713333333333</v>
       </c>
       <c r="Q171" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="172" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -9812,7 +9812,7 @@
         <v>502353.41100000002</v>
       </c>
       <c r="E172" s="5">
-        <v>0</v>
+        <v>524392.65100000007</v>
       </c>
       <c r="F172" s="5">
         <v>0</v>
@@ -9842,13 +9842,13 @@
         <v>0</v>
       </c>
       <c r="O172" s="16">
-        <v>1091889.5924789999</v>
+        <v>1616282.2434789999</v>
       </c>
       <c r="P172" s="17">
-        <v>545944.79623949993</v>
+        <v>538760.74782633339</v>
       </c>
       <c r="Q172" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="173" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -9862,7 +9862,7 @@
         <v>13266.02</v>
       </c>
       <c r="E173" s="5">
-        <v>0</v>
+        <v>721624</v>
       </c>
       <c r="F173" s="5">
         <v>0</v>
@@ -9892,10 +9892,10 @@
         <v>0</v>
       </c>
       <c r="O173" s="16">
-        <v>24784.87</v>
+        <v>746408.87</v>
       </c>
       <c r="P173" s="17">
-        <v>12392.434999999999</v>
+        <v>248802.95666666667</v>
       </c>
       <c r="Q173" s="18" t="s">
         <v>25</v>
@@ -9912,7 +9912,7 @@
         <v>32120</v>
       </c>
       <c r="E174" s="5">
-        <v>0</v>
+        <v>28640</v>
       </c>
       <c r="F174" s="5">
         <v>0</v>
@@ -9942,13 +9942,13 @@
         <v>0</v>
       </c>
       <c r="O174" s="16">
-        <v>62440</v>
+        <v>91080</v>
       </c>
       <c r="P174" s="17">
-        <v>31220</v>
+        <v>30360</v>
       </c>
       <c r="Q174" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="175" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -9962,7 +9962,7 @@
         <v>296551.63</v>
       </c>
       <c r="E175" s="5">
-        <v>0</v>
+        <v>198631.04000000001</v>
       </c>
       <c r="F175" s="5">
         <v>0</v>
@@ -9992,10 +9992,10 @@
         <v>0</v>
       </c>
       <c r="O175" s="16">
-        <v>702700.12</v>
+        <v>901331.16</v>
       </c>
       <c r="P175" s="17">
-        <v>351350.06</v>
+        <v>300443.72000000003</v>
       </c>
       <c r="Q175" s="18" t="s">
         <v>24</v>
@@ -10012,7 +10012,7 @@
         <v>18788</v>
       </c>
       <c r="E176" s="5">
-        <v>0</v>
+        <v>43159</v>
       </c>
       <c r="F176" s="5">
         <v>0</v>
@@ -10042,13 +10042,13 @@
         <v>0</v>
       </c>
       <c r="O176" s="16">
-        <v>50443.32</v>
+        <v>93602.32</v>
       </c>
       <c r="P176" s="17">
-        <v>25221.66</v>
+        <v>31200.773333333334</v>
       </c>
       <c r="Q176" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="177" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10062,7 +10062,7 @@
         <v>282849.81</v>
       </c>
       <c r="E177" s="5">
-        <v>0</v>
+        <v>384646.24</v>
       </c>
       <c r="F177" s="5">
         <v>0</v>
@@ -10092,13 +10092,13 @@
         <v>0</v>
       </c>
       <c r="O177" s="16">
-        <v>707576.42500000005</v>
+        <v>1092222.665</v>
       </c>
       <c r="P177" s="17">
-        <v>353788.21250000002</v>
+        <v>364074.22166666662</v>
       </c>
       <c r="Q177" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="178" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10112,7 +10112,7 @@
         <v>64280</v>
       </c>
       <c r="E178" s="5">
-        <v>0</v>
+        <v>78893</v>
       </c>
       <c r="F178" s="5">
         <v>0</v>
@@ -10142,13 +10142,13 @@
         <v>0</v>
       </c>
       <c r="O178" s="16">
-        <v>156097.60999999999</v>
+        <v>234990.61</v>
       </c>
       <c r="P178" s="17">
-        <v>78048.804999999993</v>
+        <v>78330.203333333324</v>
       </c>
       <c r="Q178" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="179" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10162,7 +10162,7 @@
         <v>293076</v>
       </c>
       <c r="E179" s="5">
-        <v>0</v>
+        <v>688047.95600000001</v>
       </c>
       <c r="F179" s="5">
         <v>0</v>
@@ -10192,13 +10192,13 @@
         <v>0</v>
       </c>
       <c r="O179" s="16">
-        <v>1050125.81</v>
+        <v>1738173.7660000001</v>
       </c>
       <c r="P179" s="17">
-        <v>525062.90500000003</v>
+        <v>579391.25533333339</v>
       </c>
       <c r="Q179" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="180" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10212,7 +10212,7 @@
         <v>101660</v>
       </c>
       <c r="E180" s="5">
-        <v>0</v>
+        <v>344250</v>
       </c>
       <c r="F180" s="5">
         <v>0</v>
@@ -10242,10 +10242,10 @@
         <v>0</v>
       </c>
       <c r="O180" s="16">
-        <v>197290</v>
+        <v>541540</v>
       </c>
       <c r="P180" s="17">
-        <v>98645</v>
+        <v>180513.33333333334</v>
       </c>
       <c r="Q180" s="18" t="s">
         <v>25</v>
@@ -10262,7 +10262,7 @@
         <v>8124.98</v>
       </c>
       <c r="E181" s="5">
-        <v>0</v>
+        <v>9938.08</v>
       </c>
       <c r="F181" s="5">
         <v>0</v>
@@ -10292,16 +10292,16 @@
         <v>0</v>
       </c>
       <c r="O181" s="16">
-        <v>21084.720000000001</v>
+        <v>31022.800000000003</v>
       </c>
       <c r="P181" s="17">
-        <v>10542.36</v>
+        <v>10340.933333333334</v>
       </c>
       <c r="Q181" s="18" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="182" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="182" spans="2:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B182" s="15" t="s">
         <v>18</v>
       </c>
@@ -10345,10 +10345,10 @@
         <v>226000</v>
       </c>
       <c r="P182" s="17">
-        <v>113000</v>
+        <v>75333.333333333328</v>
       </c>
       <c r="Q182" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="183" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10362,7 +10362,7 @@
         <v>308280</v>
       </c>
       <c r="E183" s="5">
-        <v>0</v>
+        <v>308080</v>
       </c>
       <c r="F183" s="5">
         <v>0</v>
@@ -10392,10 +10392,10 @@
         <v>0</v>
       </c>
       <c r="O183" s="16">
-        <v>616560</v>
+        <v>924640</v>
       </c>
       <c r="P183" s="17">
-        <v>308280</v>
+        <v>308213.33333333331</v>
       </c>
       <c r="Q183" s="18" t="s">
         <v>24</v>
@@ -10412,7 +10412,7 @@
         <v>0</v>
       </c>
       <c r="E184" s="5">
-        <v>0</v>
+        <v>33000</v>
       </c>
       <c r="F184" s="5">
         <v>0</v>
@@ -10442,13 +10442,13 @@
         <v>0</v>
       </c>
       <c r="O184" s="16">
-        <v>22200</v>
+        <v>55200</v>
       </c>
       <c r="P184" s="17">
-        <v>11100</v>
+        <v>18400</v>
       </c>
       <c r="Q184" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="185" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10462,7 +10462,7 @@
         <v>4875</v>
       </c>
       <c r="E185" s="5">
-        <v>0</v>
+        <v>13124.353999999999</v>
       </c>
       <c r="F185" s="5">
         <v>0</v>
@@ -10492,13 +10492,13 @@
         <v>0</v>
       </c>
       <c r="O185" s="16">
-        <v>8437.5000089999994</v>
+        <v>21561.854008999999</v>
       </c>
       <c r="P185" s="17">
-        <v>4218.7500044999997</v>
+        <v>7187.2846696666666</v>
       </c>
       <c r="Q185" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="186" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10512,7 +10512,7 @@
         <v>65297.9</v>
       </c>
       <c r="E186" s="5">
-        <v>0</v>
+        <v>127145.85</v>
       </c>
       <c r="F186" s="5">
         <v>0</v>
@@ -10542,13 +10542,13 @@
         <v>0</v>
       </c>
       <c r="O186" s="16">
-        <v>201655.484991</v>
+        <v>328801.33499100001</v>
       </c>
       <c r="P186" s="17">
-        <v>100827.7424955</v>
+        <v>109600.444997</v>
       </c>
       <c r="Q186" s="18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="187" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10562,7 +10562,7 @@
         <v>30222.359</v>
       </c>
       <c r="E187" s="5">
-        <v>0</v>
+        <v>16574.118999999999</v>
       </c>
       <c r="F187" s="5">
         <v>0</v>
@@ -10592,10 +10592,10 @@
         <v>0</v>
       </c>
       <c r="O187" s="16">
-        <v>72587.867521000007</v>
+        <v>89161.986521000013</v>
       </c>
       <c r="P187" s="17">
-        <v>36293.933760500004</v>
+        <v>29720.662173666671</v>
       </c>
       <c r="Q187" s="18" t="s">
         <v>24</v>
@@ -10612,7 +10612,7 @@
         <v>582743.38</v>
       </c>
       <c r="E188" s="5">
-        <v>0</v>
+        <v>375415.49</v>
       </c>
       <c r="F188" s="5">
         <v>0</v>
@@ -10642,13 +10642,13 @@
         <v>0</v>
       </c>
       <c r="O188" s="16">
-        <v>731531.74</v>
+        <v>1106947.23</v>
       </c>
       <c r="P188" s="17">
-        <v>365765.87</v>
+        <v>368982.41</v>
       </c>
       <c r="Q188" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="189" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10695,10 +10695,10 @@
         <v>349265</v>
       </c>
       <c r="P189" s="17">
-        <v>174632.5</v>
+        <v>116421.66666666667</v>
       </c>
       <c r="Q189" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="190" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10712,7 +10712,7 @@
         <v>1000</v>
       </c>
       <c r="E190" s="5">
-        <v>0</v>
+        <v>1849.0139999999999</v>
       </c>
       <c r="F190" s="5">
         <v>0</v>
@@ -10742,10 +10742,10 @@
         <v>0</v>
       </c>
       <c r="O190" s="16">
-        <v>1000</v>
+        <v>2849.0140000000001</v>
       </c>
       <c r="P190" s="17">
-        <v>500</v>
+        <v>949.67133333333334</v>
       </c>
       <c r="Q190" s="18" t="s">
         <v>25</v>
@@ -10762,7 +10762,7 @@
         <v>176627.3</v>
       </c>
       <c r="E191" s="5">
-        <v>0</v>
+        <v>152263.59</v>
       </c>
       <c r="F191" s="5">
         <v>0</v>
@@ -10792,13 +10792,13 @@
         <v>0</v>
       </c>
       <c r="O191" s="16">
-        <v>332582.5</v>
+        <v>484846.08999999997</v>
       </c>
       <c r="P191" s="17">
-        <v>166291.25</v>
+        <v>161615.36333333334</v>
       </c>
       <c r="Q191" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="192" spans="2:17" ht="13.35" customHeight="1" x14ac:dyDescent="0.2">
@@ -10809,10 +10809,10 @@
         <v>329126.52999999997</v>
       </c>
       <c r="D192" s="5">
-        <v>391154.06</v>
+        <v>354485.06</v>
       </c>
       <c r="E192" s="5">
-        <v>0</v>
+        <v>539901.51</v>
       </c>
       <c r="F192" s="5">
         <v>0</v>
@@ -10842,10 +10842,10 @@
         <v>0</v>
       </c>
       <c r="O192" s="16">
-        <v>720280.59</v>
+        <v>1223513.1000000001</v>
       </c>
       <c r="P192" s="17">
-        <v>360140.29499999998</v>
+        <v>407837.7</v>
       </c>
       <c r="Q192" s="18" t="s">
         <v>25</v>
@@ -10898,7 +10898,7 @@
         <v>0</v>
       </c>
       <c r="Q193" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="194" spans="2:17" ht="13.35" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -10909,10 +10909,10 @@
         <v>3839057.96</v>
       </c>
       <c r="D194" s="8">
-        <v>3660413.09</v>
+        <v>3623744.09</v>
       </c>
       <c r="E194" s="8">
-        <v>0</v>
+        <v>4695972.1340000005</v>
       </c>
       <c r="F194" s="8">
         <v>0</v>
@@ -10942,10 +10942,10 @@
         <v>0</v>
       </c>
       <c r="O194" s="25">
-        <v>7499471.0499999998</v>
+        <v>12158774.184</v>
       </c>
       <c r="P194" s="26">
-        <v>3749735.5249999999</v>
+        <v>4052924.7280000006</v>
       </c>
       <c r="Q194" s="27"/>
     </row>

</xml_diff>